<commit_message>
avances 15/10 tema objetos
</commit_message>
<xml_diff>
--- a/Arrays/pruebasEscritorioArreglos.xlsx
+++ b/Arrays/pruebasEscritorioArreglos.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ejercicios\Ejercicios_clase_miguel\Arrays\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A886ABE-51AE-477F-A780-D7454EF62F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F06D10-9AE6-44F9-8A89-BF9EB24DB682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{3B066930-FAA7-41EA-8A91-1C0FE1B87CDD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{3B066930-FAA7-41EA-8A91-1C0FE1B87CDD}"/>
   </bookViews>
   <sheets>
     <sheet name="Ejercicio 1" sheetId="1" r:id="rId1"/>
     <sheet name="Ejercicio 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Ejercicio 3" sheetId="3" r:id="rId3"/>
+    <sheet name="Ejercicio 4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="96">
   <si>
     <t>Cantidad de productos</t>
   </si>
@@ -103,6 +105,231 @@
   </si>
   <si>
     <t>3. café</t>
+  </si>
+  <si>
+    <t>ingreo los numeros</t>
+  </si>
+  <si>
+    <t>nota</t>
+  </si>
+  <si>
+    <t>leernotavalida()</t>
+  </si>
+  <si>
+    <t>nota &gt;= 0 and nota &lt;=5</t>
+  </si>
+  <si>
+    <t>while true</t>
+  </si>
+  <si>
+    <t>break</t>
+  </si>
+  <si>
+    <t>push numeros</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>total / numeros</t>
+  </si>
+  <si>
+    <t>unircomas()</t>
+  </si>
+  <si>
+    <t>calcularPromedio()</t>
+  </si>
+  <si>
+    <t>texto</t>
+  </si>
+  <si>
+    <t>prmedioAprobado</t>
+  </si>
+  <si>
+    <t>promedio &gt;= 3.0</t>
+  </si>
+  <si>
+    <t>i &lt;= 5</t>
+  </si>
+  <si>
+    <t>[4,5]</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>preguntamos</t>
+  </si>
+  <si>
+    <t>[4.5, 3]</t>
+  </si>
+  <si>
+    <t>[4.5, 3, 2.5]</t>
+  </si>
+  <si>
+    <t>[4.5, 3, 2.5, 4]</t>
+  </si>
+  <si>
+    <t>3.5</t>
+  </si>
+  <si>
+    <t>[4.5, 3, 2.5, 4, 3.5]</t>
+  </si>
+  <si>
+    <t>total+=[i]</t>
+  </si>
+  <si>
+    <t>i&lt;5</t>
+  </si>
+  <si>
+    <t>""</t>
+  </si>
+  <si>
+    <t>i==0</t>
+  </si>
+  <si>
+    <t>text == [i]</t>
+  </si>
+  <si>
+    <t>4.5, 3</t>
+  </si>
+  <si>
+    <t>4.5, 3, 2.5</t>
+  </si>
+  <si>
+    <t>4.5, 3, 2.5, 4</t>
+  </si>
+  <si>
+    <t>text += ", " [i]</t>
+  </si>
+  <si>
+    <t>4.5,  3,  2.5,  4.3, 4</t>
+  </si>
+  <si>
+    <t>cantidad N</t>
+  </si>
+  <si>
+    <t>leernumeros()</t>
+  </si>
+  <si>
+    <t>ingresar numero</t>
+  </si>
+  <si>
+    <t>push numero</t>
+  </si>
+  <si>
+    <t>array numeros</t>
+  </si>
+  <si>
+    <t>obtenerultimo()</t>
+  </si>
+  <si>
+    <t>array.length -1</t>
+  </si>
+  <si>
+    <t>mostrarMedio()</t>
+  </si>
+  <si>
+    <t>tamaño array</t>
+  </si>
+  <si>
+    <t>if tamaño %2 == 0</t>
+  </si>
+  <si>
+    <t>i&lt;=cantidad N</t>
+  </si>
+  <si>
+    <t>[8]</t>
+  </si>
+  <si>
+    <t>[8, 3]</t>
+  </si>
+  <si>
+    <t>[8, 4, 9]</t>
+  </si>
+  <si>
+    <t>[8, 4, 9, 1]</t>
+  </si>
+  <si>
+    <t>[8, 4, 9, 1, 7]</t>
+  </si>
+  <si>
+    <t>else [tamaño]</t>
+  </si>
+  <si>
+    <t>dias</t>
+  </si>
+  <si>
+    <t>["Lunes", "Martes", "Miércoles", "Jueves", "Viernes", "Sábado", "Domingo"]</t>
+  </si>
+  <si>
+    <t>leerventas()</t>
+  </si>
+  <si>
+    <t>i &lt; dias.length</t>
+  </si>
+  <si>
+    <t>push ventas</t>
+  </si>
+  <si>
+    <t>calculartotal()</t>
+  </si>
+  <si>
+    <t>i &lt; numeros.length</t>
+  </si>
+  <si>
+    <t>suma += numero[i]</t>
+  </si>
+  <si>
+    <t>mostrarreporte()</t>
+  </si>
+  <si>
+    <t>i&lt;dias.length</t>
+  </si>
+  <si>
+    <t>console.log</t>
+  </si>
+  <si>
+    <t>[120000]</t>
+  </si>
+  <si>
+    <t>[120000, 95000]</t>
+  </si>
+  <si>
+    <t>[120000, 95000, 110000]</t>
+  </si>
+  <si>
+    <t>[120000, 95000, 110000, 130000]</t>
+  </si>
+  <si>
+    <t>[120000, 95000, 110000, 130000, 210000]</t>
+  </si>
+  <si>
+    <t>[120000, 95000, 110000, 130000, 210000, 260000]</t>
+  </si>
+  <si>
+    <t>[120000, 95000, 110000, 130000, 210000, 260000, 180000]</t>
+  </si>
+  <si>
+    <t>lunes: 120000</t>
+  </si>
+  <si>
+    <t>martes: 95000</t>
+  </si>
+  <si>
+    <t>miercoles: 110000</t>
+  </si>
+  <si>
+    <t>jueves: 130000</t>
+  </si>
+  <si>
+    <t>viernes: 210000</t>
+  </si>
+  <si>
+    <t>sabado: 260000</t>
+  </si>
+  <si>
+    <t>domingo: 180000</t>
   </si>
 </sst>
 </file>
@@ -138,10 +365,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -642,9 +872,1351 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C555D62-1BFE-4C95-9707-B69EA68F0C86}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:S21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M1" t="s">
+        <v>30</v>
+      </c>
+      <c r="S1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" t="s">
+        <v>32</v>
+      </c>
+      <c r="N2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O2" t="s">
+        <v>45</v>
+      </c>
+      <c r="P2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>48</v>
+      </c>
+      <c r="R2" t="s">
+        <v>52</v>
+      </c>
+      <c r="S2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>4.5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>37</v>
+      </c>
+      <c r="O3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
+        <v>37</v>
+      </c>
+      <c r="S3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" t="s">
+        <v>37</v>
+      </c>
+      <c r="O4" t="s">
+        <v>37</v>
+      </c>
+      <c r="P4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R4" t="s">
+        <v>37</v>
+      </c>
+      <c r="S4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" t="s">
+        <v>37</v>
+      </c>
+      <c r="O5" t="s">
+        <v>37</v>
+      </c>
+      <c r="P5" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R5" t="s">
+        <v>37</v>
+      </c>
+      <c r="S5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>2.5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" t="s">
+        <v>37</v>
+      </c>
+      <c r="L6" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" t="s">
+        <v>37</v>
+      </c>
+      <c r="O6" t="s">
+        <v>37</v>
+      </c>
+      <c r="P6" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>37</v>
+      </c>
+      <c r="R6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K7" t="s">
+        <v>37</v>
+      </c>
+      <c r="L7" t="s">
+        <v>37</v>
+      </c>
+      <c r="M7" t="s">
+        <v>37</v>
+      </c>
+      <c r="N7" t="s">
+        <v>37</v>
+      </c>
+      <c r="O7" t="s">
+        <v>37</v>
+      </c>
+      <c r="P7" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>37</v>
+      </c>
+      <c r="R7" t="s">
+        <v>37</v>
+      </c>
+      <c r="S7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" t="s">
+        <v>37</v>
+      </c>
+      <c r="K8" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8" t="s">
+        <v>37</v>
+      </c>
+      <c r="M8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N8" t="s">
+        <v>37</v>
+      </c>
+      <c r="O8" t="s">
+        <v>37</v>
+      </c>
+      <c r="P8" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>37</v>
+      </c>
+      <c r="R8" t="s">
+        <v>37</v>
+      </c>
+      <c r="S8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9" t="s">
+        <v>10</v>
+      </c>
+      <c r="K9">
+        <v>4.5</v>
+      </c>
+      <c r="L9" t="s">
+        <v>37</v>
+      </c>
+      <c r="M9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N9" t="s">
+        <v>37</v>
+      </c>
+      <c r="O9" t="s">
+        <v>37</v>
+      </c>
+      <c r="P9" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>37</v>
+      </c>
+      <c r="R9" t="s">
+        <v>37</v>
+      </c>
+      <c r="S9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="H10">
+        <v>4.5</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10" t="s">
+        <v>10</v>
+      </c>
+      <c r="K10">
+        <v>7.5</v>
+      </c>
+      <c r="L10" t="s">
+        <v>37</v>
+      </c>
+      <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
+        <v>37</v>
+      </c>
+      <c r="O10" t="s">
+        <v>37</v>
+      </c>
+      <c r="P10" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>37</v>
+      </c>
+      <c r="R10" t="s">
+        <v>37</v>
+      </c>
+      <c r="S10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="H11">
+        <v>7.5</v>
+      </c>
+      <c r="I11">
+        <v>2</v>
+      </c>
+      <c r="J11" t="s">
+        <v>10</v>
+      </c>
+      <c r="K11">
+        <v>10</v>
+      </c>
+      <c r="L11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M11" t="s">
+        <v>37</v>
+      </c>
+      <c r="N11" t="s">
+        <v>37</v>
+      </c>
+      <c r="O11" t="s">
+        <v>37</v>
+      </c>
+      <c r="P11" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>37</v>
+      </c>
+      <c r="R11" t="s">
+        <v>37</v>
+      </c>
+      <c r="S11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="H12">
+        <v>10</v>
+      </c>
+      <c r="I12">
+        <v>3</v>
+      </c>
+      <c r="J12" t="s">
+        <v>10</v>
+      </c>
+      <c r="K12">
+        <v>14</v>
+      </c>
+      <c r="L12" t="s">
+        <v>37</v>
+      </c>
+      <c r="M12" t="s">
+        <v>37</v>
+      </c>
+      <c r="N12" t="s">
+        <v>37</v>
+      </c>
+      <c r="O12" t="s">
+        <v>37</v>
+      </c>
+      <c r="P12" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>37</v>
+      </c>
+      <c r="R12" t="s">
+        <v>37</v>
+      </c>
+      <c r="S12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="H13">
+        <v>14</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+      <c r="J13" t="s">
+        <v>10</v>
+      </c>
+      <c r="K13">
+        <v>17.5</v>
+      </c>
+      <c r="L13" t="s">
+        <v>37</v>
+      </c>
+      <c r="M13" t="s">
+        <v>37</v>
+      </c>
+      <c r="N13" t="s">
+        <v>37</v>
+      </c>
+      <c r="O13" t="s">
+        <v>37</v>
+      </c>
+      <c r="P13" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>37</v>
+      </c>
+      <c r="R13" t="s">
+        <v>37</v>
+      </c>
+      <c r="S13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="H14">
+        <v>17.5</v>
+      </c>
+      <c r="I14">
+        <v>5</v>
+      </c>
+      <c r="J14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" t="s">
+        <v>37</v>
+      </c>
+      <c r="L14">
+        <v>3.5</v>
+      </c>
+      <c r="M14" t="s">
+        <v>37</v>
+      </c>
+      <c r="N14" t="s">
+        <v>37</v>
+      </c>
+      <c r="O14" t="s">
+        <v>37</v>
+      </c>
+      <c r="P14" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>37</v>
+      </c>
+      <c r="R14" t="s">
+        <v>37</v>
+      </c>
+      <c r="S14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I15" t="s">
+        <v>37</v>
+      </c>
+      <c r="J15" t="s">
+        <v>37</v>
+      </c>
+      <c r="K15" t="s">
+        <v>37</v>
+      </c>
+      <c r="L15" t="s">
+        <v>37</v>
+      </c>
+      <c r="M15" t="s">
+        <v>46</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15" t="s">
+        <v>10</v>
+      </c>
+      <c r="P15" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q15">
+        <v>4.5</v>
+      </c>
+      <c r="R15" t="s">
+        <v>37</v>
+      </c>
+      <c r="S15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="N16">
+        <v>1</v>
+      </c>
+      <c r="O16" t="s">
+        <v>10</v>
+      </c>
+      <c r="P16" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>37</v>
+      </c>
+      <c r="R16" t="s">
+        <v>49</v>
+      </c>
+      <c r="S16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="13:19" x14ac:dyDescent="0.25">
+      <c r="N17">
+        <v>2</v>
+      </c>
+      <c r="O17" t="s">
+        <v>10</v>
+      </c>
+      <c r="P17" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>37</v>
+      </c>
+      <c r="R17" t="s">
+        <v>50</v>
+      </c>
+      <c r="S17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="13:19" x14ac:dyDescent="0.25">
+      <c r="N18">
+        <v>3</v>
+      </c>
+      <c r="O18" t="s">
+        <v>10</v>
+      </c>
+      <c r="P18" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>37</v>
+      </c>
+      <c r="R18" t="s">
+        <v>51</v>
+      </c>
+      <c r="S18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="13:19" x14ac:dyDescent="0.25">
+      <c r="N19">
+        <v>4</v>
+      </c>
+      <c r="O19" t="s">
+        <v>10</v>
+      </c>
+      <c r="P19" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>37</v>
+      </c>
+      <c r="R19" t="s">
+        <v>53</v>
+      </c>
+      <c r="S19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="13:19" x14ac:dyDescent="0.25">
+      <c r="M20" t="s">
+        <v>53</v>
+      </c>
+      <c r="N20">
+        <v>5</v>
+      </c>
+      <c r="O20" t="s">
+        <v>17</v>
+      </c>
+      <c r="P20" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>37</v>
+      </c>
+      <c r="R20" t="s">
+        <v>37</v>
+      </c>
+      <c r="S20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="13:19" x14ac:dyDescent="0.25">
+      <c r="S21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{132DFF67-149E-4B2E-B03F-3F46D8AF3B15}">
+  <dimension ref="B1:K10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I2" t="s">
+        <v>62</v>
+      </c>
+      <c r="J2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7">
+        <v>7</v>
+      </c>
+      <c r="F7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>69</v>
+      </c>
+      <c r="H8" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" t="s">
+        <v>37</v>
+      </c>
+      <c r="K8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="H9">
+        <v>7</v>
+      </c>
+      <c r="I9" t="s">
+        <v>37</v>
+      </c>
+      <c r="J9" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I10">
+        <v>5</v>
+      </c>
+      <c r="J10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K10">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E8F8998-1182-4717-9EA4-319C33C186CB}">
+  <dimension ref="B1:K26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" ht="105" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="105" x14ac:dyDescent="0.25">
+      <c r="C9">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12">
+        <v>215000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13">
+        <v>425000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14">
+        <v>555000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="F15">
+        <v>4</v>
+      </c>
+      <c r="G15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15">
+        <v>765000</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="F16">
+        <v>5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16">
+        <v>825000</v>
+      </c>
+    </row>
+    <row r="17" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F17">
+        <v>6</v>
+      </c>
+      <c r="G17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17">
+        <v>1105000</v>
+      </c>
+    </row>
+    <row r="18" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <v>7</v>
+      </c>
+      <c r="G18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19" t="s">
+        <v>10</v>
+      </c>
+      <c r="K19" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20" t="s">
+        <v>10</v>
+      </c>
+      <c r="K20" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="21" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="I21">
+        <v>2</v>
+      </c>
+      <c r="J21" t="s">
+        <v>10</v>
+      </c>
+      <c r="K21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="I22">
+        <v>3</v>
+      </c>
+      <c r="J22" t="s">
+        <v>10</v>
+      </c>
+      <c r="K22" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="I23">
+        <v>4</v>
+      </c>
+      <c r="J23" t="s">
+        <v>10</v>
+      </c>
+      <c r="K23" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="24" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="I24">
+        <v>5</v>
+      </c>
+      <c r="J24" t="s">
+        <v>10</v>
+      </c>
+      <c r="K24" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="I25">
+        <v>6</v>
+      </c>
+      <c r="J25" t="s">
+        <v>10</v>
+      </c>
+      <c r="K25" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="I26">
+        <v>7</v>
+      </c>
+      <c r="J26" t="s">
+        <v>17</v>
+      </c>
+      <c r="K26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>